<commit_message>
Add Chelsea Dagger and Shoot to Thrill to Between Whistles
Imported from the song-submission form via scripts/import_songs_tsv.py:

  Chelsea dagger    starts 3:06 (requested by Ken)
  Shoot to Thrill   starts 1:02 (requested by Kelly)

Between Whistles goes from 15 to 17 tracks; 27 to 29 overall. Regenerates
wild-hockey-songs.xlsx to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XcB6P62pe2uNn5vjS1vRK
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -839,232 +839,276 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Thunderstruck</t>
+          <t>Chelsea dagger</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+          <t>https://open.spotify.com/track/0txisWocI2H8yPRjYxLo83</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>2:38</t>
+          <t>3:06</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>Shoot to Thrill</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+          <t>https://open.spotify.com/track/0C80GCp0mMuBzLf3EAXqxv</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>1:03</t>
+          <t>1:02</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>Thunderstruck</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Goal FOR</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>0:41</t>
+          <t>2:38</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>Kickstart my Heart</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Goal FOR</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>0:46</t>
+          <t>1:03</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Fireball</t>
+          <t>Shake it Off</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Powerplay</t>
+          <t>Goal AGAINST</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>1:32</t>
+          <t>0:41</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>I Did Something Bad</t>
+          <t>We're not gonna take it</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>Goal AGAINST</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>0:46</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Bad Girls</t>
+          <t>Fireball</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
+          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>Powerplay</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
+          <t>1:32</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Final Countdown</t>
+          <t>I Did Something Bad</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>Penalty Kill</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>4:08</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Knights of Cydonia</t>
+          <t>Bad Girls</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>Penalty Kill</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>4:10</t>
+          <t>1:33</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Final Countdown</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>End Game Intensity</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Knights of Cydonia</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>End Game Intensity</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Immigrant Song</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>End Game Intensity</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>0:01</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.TRACKS block in index.html. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D28"/>
+  <autoFilter ref="A1:D30"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1093,6 +1137,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 10 songs to Between Whistles; add permission allowlist
Imports a 10-song batch from the submission sheet via
scripts/import_songs_tsv.py. Three rows spelled the category "Whitles";
corrected to "Whistles" before importing, since the same batch spells it
correctly on the other seven rows.

Between Whistles goes from 17 to 27 tracks; 29 to 39 overall. Regenerates
wild-hockey-songs.xlsx to match.

Also adds .claude/settings.json with a permissions allowlist for the
read-only and repo-pinned calls used repeatedly in this workflow, so they
stop prompting on every run. Committed rather than left local so it
survives fresh checkouts.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XcB6P62pe2uNn5vjS1vRK
</commit_message>
<xml_diff>
--- a/wild-hockey-songs.xlsx
+++ b/wild-hockey-songs.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Songs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Songs'!$A$1:$D$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -883,232 +883,448 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Thunderstruck</t>
+          <t>9 to 5</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+          <t>https://open.spotify.com/track/4w3tQBXhn5345eUXDGBWZG</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2:38</t>
+          <t>1:28</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Kickstart my Heart</t>
+          <t>Lush Life</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+          <t>https://open.spotify.com/track/0e6WPtkB9dwFiwspkEeen2</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Goal FOR</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>1:03</t>
+          <t>0:49</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Shake it Off</t>
+          <t>pink pony club</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+          <t>https://open.spotify.com/track/1k2pQc5i348DCHwbn5KTdc</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>0:41</t>
+          <t>2:15</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>We're not gonna take it</t>
+          <t>the distance</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+          <t>https://open.spotify.com/track/1szwDbVdIdoQq5mG5GXAmJ</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Goal AGAINST</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>0:46</t>
+          <t>0:42</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Fireball</t>
+          <t>wild thing</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+          <t>https://open.spotify.com/track/01lZlV0coZWuhzZpFQZ43u</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Powerplay</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>1:32</t>
-        </is>
-      </c>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>I Did Something Bad</t>
+          <t>brass</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+          <t>https://open.spotify.com/track/03ZyPqIZXdBNNVIpM2KORq</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>0:44</t>
+          <t>0:30</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Bad Girls</t>
+          <t>get ready for this</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
+          <t>https://open.spotify.com/track/5zyxpZ8xZmTuhXOuZq4KBG</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Penalty Kill</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>1:33</t>
+          <t>0:25</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Final Countdown</t>
+          <t>handclap</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+          <t>https://open.spotify.com/track/0y3fi7fknIXOxnkbUgzT3n</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>4:08</t>
+          <t>0:27</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Knights of Cydonia</t>
+          <t>rock n roll gary glitter</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+          <t>https://open.spotify.com/track/1t3mzpCfaMsEqL1Fbq46ST</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>End Game Intensity</t>
+          <t>Between Whistles</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>4:10</t>
+          <t>0:44</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>legend</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3SWqGa1J0M7hSBUDM0KePD</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Between Whistles</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>0:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Thunderstruck</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/57bgtoPSgt236HzfBOd8kj</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Goal FOR</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>2:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Kickstart my Heart</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1ZipIhmm5baGBobKoAFWHE</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Goal FOR</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>1:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Shake it Off</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3pv7Q5v2dpdefwdWIvE7yH</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Goal AGAINST</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>0:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>We're not gonna take it</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/5X79VgaOn8pDTpTKu3PixN</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Goal AGAINST</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>0:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Fireball</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4Y7XAxTANhu3lmnLAzhWJW</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Powerplay</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>1:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>I Did Something Bad</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/4svZDCRz4cJoneBpjpx8DJ</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>0:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Bad Girls</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/1ibRqifchaAfeNdQGpbRVW</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Penalty Kill</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>1:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Final Countdown</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/3MrRksHupTVEQ7YbA0FsZK</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>End Game Intensity</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>4:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Knights of Cydonia</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>https://open.spotify.com/track/7ouMYWpwJ422jRcDASZB7P</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>End Game Intensity</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>4:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>Immigrant Song</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>https://open.spotify.com/track/78lgmZwycJ3nzsdgmPPGNx</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>End Game Intensity</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>0:01</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>Exported from the window.TRACKS block in index.html. Start Time is shown as m:ss and corresponds to the startSec value (in seconds); a blank means the track plays from the beginning.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D30"/>
+  <autoFilter ref="A1:D40"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1139,6 +1355,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId39"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>